<commit_message>
Update style assignment spreadsheet for revised plain-language script
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HRvtTA56nnGLFzY4MmhFZG
</commit_message>
<xml_diff>
--- a/script-style-plan/台本スタイル割り.xlsx
+++ b/script-style-plan/台本スタイル割り.xlsx
@@ -692,7 +692,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>周囲を何万人もの見知らぬ他人が行き交う場所で、人はどこまで無防備になれるだろうか。</t>
+          <t>たくさんの人が行き交う駅のど真ん中で、服を脱ぐなんて絶対にあり得ないと思いますよね。</t>
         </is>
       </c>
       <c r="D2" s="2">
@@ -725,10 +725,14 @@
       <c r="J2" s="7" t="n"/>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>真上から見た駅コンコース。無数の点（人）が流れる中、中央の1人だけが立ち止まる。「無防備」の文字がゆっくり浮かぶ。</t>
-        </is>
-      </c>
-      <c r="L2" s="3" t="n"/>
+          <t>真上から見た駅コンコース。無数の点（人）が流れる中、中央の1人だけが立ち止まる。「絶対にあり得ない」の文字が浮かぶ。</t>
+        </is>
+      </c>
+      <c r="L2" s="8" t="inlineStr">
+        <is>
+          <t>服を脱ぐ場面は描かない。人物は棒人間のまま、言葉だけで伝える。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -741,7 +745,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>群衆のど真ん中にある四角い箱に足を踏み入れた瞬間、私たちの脳は奇妙な錯誤を起こす。</t>
+          <t>でも、たった畳1枚分の小さな箱に入るだけで、人間の脳は信じられない勘違いを起こしてしまいます。</t>
         </is>
       </c>
       <c r="D3" s="2">
@@ -774,7 +778,7 @@
       <c r="J3" s="7" t="n"/>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>点の流れの中央に黒いキューブが出現。人物が入った瞬間、画面全体が一瞬グリッチして「錯誤」と表示。</t>
+          <t>点の流れの中央に黒いキューブが出現（「畳1枚分」の寸法線を添える）。人物が入った瞬間、画面が一瞬グリッチして「勘違い」と表示。</t>
         </is>
       </c>
       <c r="L3" s="3" t="n"/>
@@ -790,7 +794,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026年9月、首都圏の主要ターミナル駅に設置されたテレワーク用防音個室ブース「ステーションポッド」内で、利用者が衣服を脱ぎ捨てて外部に露出する不適切行為の動画がSNSに拡散され、警察が捜査に乗り出す騒動へと発展した。</t>
+          <t>2026年9月、都内の大きな駅に置かれたテレワーク用の防音個室「ステーションポッド」の中で、服を脱いで外に見せびらかすような動画がネットに広まり、警察が動く大きな騒ぎになりました。</t>
         </is>
       </c>
       <c r="D4" s="2">
@@ -823,12 +827,12 @@
       <c r="J4" s="7" t="n"/>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>暗く抑えたシェーダー背景の上に、ニュース見出し風カードと架空のSNS通知UIが積み重なる。「2026年9月」「警察が捜査」を強調。</t>
+          <t>暗く抑えたシェーダー背景の上に、ニュース見出し風カードと架空のSNS通知UIが積み重なる。「2026年9月」「警察が動く」を強調。</t>
         </is>
       </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>露出行為そのものは描かない（ブースの外観と通知UIだけで伝える）。実在のSNS・駅・商品名のロゴは使わない。事件の実在性は「要確認」シート参照。</t>
+          <t>行為そのものは描かない（ブースの外観と通知UIだけで伝える）。実在のSNS・駅・商品のロゴは使わない。事件の実在性は「要確認」シート参照。</t>
         </is>
       </c>
     </row>
@@ -843,7 +847,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>モラルの崩壊や利用者の異常性と切り捨てるのは容易だ。</t>
+          <t>おかしな人が自分勝手に暴れただけ、と片付けるのは簡単です。</t>
         </is>
       </c>
       <c r="D5" s="2">
@@ -872,7 +876,7 @@
       <c r="J5" s="7" t="n"/>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>群衆が1人の人物を指さす。「モラルの崩壊」「異常性」の文字にSVGの取り消し線が引かれる。</t>
+          <t>群衆が1人の人物を指さす。「おかしな人」の文字にSVGの取り消し線が引かれる。</t>
         </is>
       </c>
       <c r="L5" s="3" t="n"/>
@@ -888,7 +892,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>だが、この奇行の引き金を引いたのは、特殊な個人の狂気ではなく、現代の空間設計が人間の脳に仕掛けた認知のバグである。</t>
+          <t>だが、このとんでもない行動を引き起こしたのは、狭い箱に入ったときに誰もが持っている心のスイッチが入ってしまったからでした。</t>
         </is>
       </c>
       <c r="D6" s="2">
@@ -915,16 +919,20 @@
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>11 ネオン・グリッチ</t>
+          <t>12 キネティック文字</t>
         </is>
       </c>
       <c r="J6" s="7" t="n"/>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>脳の断面図（線画）の中をジェネラティブなノイズが流れ、「認知のバグ」がグリッチ表示。</t>
-        </is>
-      </c>
-      <c r="L6" s="3" t="n"/>
+          <t>脳の線画の中をジェネラティブなノイズが流れ、中央のスイッチがカチッと入る。「心のスイッチ」を強調。</t>
+        </is>
+      </c>
+      <c r="L6" s="8" t="inlineStr">
+        <is>
+          <t>台本の表記：この文だけ「だが」で、ほかの「です・ます」調と合わない。「ですが」に変えると自然。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -937,7 +945,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>心理学と社会学の光を当てて解剖してみよう。</t>
+          <t>いったい私たちの頭と、普段暮らしている街の中で何が起きていたのか、一緒に解き明かしていきましょう。</t>
         </is>
       </c>
       <c r="D7" s="2">
@@ -970,7 +978,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>タイトルカード。「心理学 × 社会学」が一筆書きで描かれ、光が走る。</t>
+          <t>タイトルカード。「頭の中 × 街の仕組み」が一筆書きで描かれ、光が走る。</t>
         </is>
       </c>
       <c r="L7" s="3" t="n"/>
@@ -981,12 +989,12 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>① 狭い箱の安全錯覚</t>
+          <t>① 狭い箱の油断</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>なぜ人は、すぐ外を他人が歩くガラス張りの箱の中で警戒を解いてしまうのか。</t>
+          <t>なぜ人は、すぐ外を大勢の人が歩いているのに、ガラス張りの箱の中で油断してしまうのでしょうか。</t>
         </is>
       </c>
       <c r="D8" s="9">
@@ -1030,12 +1038,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>① 狭い箱の安全錯覚</t>
+          <t>① 狭い箱の油断</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>コーネル大学の環境心理学者、ゲイリーエバンスが2000年に都市住民300人を対象に行った実験がある。</t>
+          <t>アメリカのコーネル大学のゲイリーエバンスという研究者が、2000年に300人の街の人を集めて実験を行いました。</t>
         </is>
       </c>
       <c r="D9" s="2">
@@ -1079,12 +1087,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>① 狭い箱の安全錯覚</t>
+          <t>① 狭い箱の油断</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>被験者を広さの異なる部屋に隔離し、窓の外に人通りがある状況で心拍数とコルチゾール値を計測しながら複雑なパズル課題に取り組ませた。</t>
+          <t>広さが違う部屋に人を入れ、窓の外を他人が通り過ぎる様子を見せながら、ドキドキする度合いやストレスを測りつつ難しいパズルを解かせたのです。</t>
         </is>
       </c>
       <c r="D10" s="2">
@@ -1124,12 +1132,12 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>① 狭い箱の安全錯覚</t>
+          <t>① 狭い箱の油断</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>その結果、床面積が狭い空間ほど、外部の視線に対する身体的警戒反応が約40パーセント低下した。</t>
+          <t>すると、部屋が狭くなればなるほど、外から見られていることへの警戒心が約40パーセントも下がりました。</t>
         </is>
       </c>
       <c r="D11" s="2">
@@ -1158,12 +1166,12 @@
       <c r="J11" s="7" t="n"/>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>部屋の広さ別の警戒反応を棒グラフで表示。小部屋の棒が下がり「−40%」が大きく出る。</t>
+          <t>部屋の広さ別の警戒心を棒グラフで表示。小部屋の棒が下がり「−40%」が大きく出る。</t>
         </is>
       </c>
       <c r="L11" s="8" t="inlineStr">
         <is>
-          <t>数値の出典が確認できていない。グラフ化すると断定の印象が強まるので、確認後に作る。</t>
+          <t>数値の出典が確認できていない。グラフにすると確かな事実に見えるので、確認後に作る。</t>
         </is>
       </c>
     </row>
@@ -1173,12 +1181,12 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>① 狭い箱の安全錯覚</t>
+          <t>① 狭い箱の油断</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>境界線が身体に迫る狭小空間は、脳に疑似的な母親の胎内のような安全シグナルを誤認させる。</t>
+          <t>壁が体にぴったり近づく狭い部屋に入ると、人間の脳は守られていると勘違いしてしまうのです。</t>
         </is>
       </c>
       <c r="D12" s="2">
@@ -1211,7 +1219,7 @@
       <c r="J12" s="7" t="n"/>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>暖色のシェーダー。四角い壁の線が丸く変形して人物を包む。「安全」が表示され、ずれて「誤認」に変わる。</t>
+          <t>暖色のシェーダー。四角い壁の線が丸く変形して人物を包む。「守られている」が表示され、ずれて「勘違い」に変わる。</t>
         </is>
       </c>
       <c r="L12" s="3" t="n"/>
@@ -1227,7 +1235,7 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>駅の雑踏を思い出してほしい。</t>
+          <t>駅の通路を思い浮かべてみてください。</t>
         </is>
       </c>
       <c r="D13" s="9">
@@ -1260,7 +1268,7 @@
       </c>
       <c r="K13" s="10" t="inlineStr">
         <is>
-          <t>駅構内の奥行き（柱・人の層）を多層パララックスで表現。手前ほど速く人が流れる。</t>
+          <t>駅の通路の奥行き（柱・人の層）を多層パララックスで表現。手前ほど速く人が流れる。</t>
         </is>
       </c>
       <c r="L13" s="10" t="n"/>
@@ -1276,7 +1284,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>何千人もの靴音が反響し、行き交う人々の肩が触れ合う通路の脇に、わずか畳一畳ほどの黒いキューブが鎮座している。</t>
+          <t>大勢の人の足音が響き、人と人が肩をぶつけそうになりながら歩いているすぐ横に、黒くて四角い電話ボックスのような箱がポツンと立っています。</t>
         </is>
       </c>
       <c r="D14" s="2">
@@ -1309,7 +1317,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>カメラが人の流れを抜けると、通路脇に黒いキューブ。「畳一畳」の寸法線をSVGで添えてもよい。</t>
+          <t>カメラが人の流れを抜けると、通路脇に黒いキューブがポツンと立っている。</t>
         </is>
       </c>
       <c r="L14" s="3" t="n"/>
@@ -1325,7 +1333,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>防音ドアを閉めた瞬間、周囲の喧騒は低く籠もった唸り声へと遮断され、目の前には自分専用のモニターと小さなデスクだけが広がる。</t>
+          <t>重いドアをパタンと閉めた瞬間、さっきまでのうるさい音が遠くのうなり声のように消えて、目の前には自分だけの机と椅子だけが残ります。</t>
         </is>
       </c>
       <c r="D15" s="2">
@@ -1374,7 +1382,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>ほんの数センチ外側をスーツ姿の通勤客が足早に通り過ぎているにもかかわらず、指先が触れる壁の圧迫感が、外の世界をまるでスクリーンの映像のように遠ざけてしまうのだ。</t>
+          <t>ガラスのすぐ向こう側をスーツ姿の大人が早歩きで通り過ぎているのに、壁に囲まれている安心感のせいで、外の世界がまるでテレビ画面の中の出来事のように遠く感じてしまうのです。</t>
         </is>
       </c>
       <c r="D16" s="2">
@@ -1403,7 +1411,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>ブース内の人物の肩越しの視点。ガラスの外の通勤客に走査線と軽いグリッチがかかり、映像のように見える。</t>
+          <t>ブース内の人物の肩越しの視点。ガラスの外の通勤客に走査線と軽いグリッチがかかり、テレビ画面のように見える。</t>
         </is>
       </c>
       <c r="L16" s="3" t="n"/>
@@ -1419,7 +1427,7 @@
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>ここまでは個人の内側の話だ。では社会の側から同じ光景を眺めると、何が見えてくるのだろうか。</t>
+          <t>ここまでは個人の心の内側の話です。では、社会全体の仕組みからこの景色を眺めると、何が見えてくるでしょうか。</t>
         </is>
       </c>
       <c r="D17" s="9">
@@ -1448,7 +1456,7 @@
       <c r="J17" s="14" t="n"/>
       <c r="K17" s="10" t="inlineStr">
         <is>
-          <t>キューブからカメラが引いていき、駅全体、さらに街全体へ。「個人 → 社会」の文字。</t>
+          <t>キューブからカメラが引いていき、駅全体、さらに街全体へ。「心の中 → 街の仕組み」の文字。</t>
         </is>
       </c>
       <c r="L17" s="10" t="n"/>
@@ -1459,12 +1467,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>② 公共空間の細分化</t>
+          <t>② 区切られた街</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>この現象は、個人の錯覚にとどまらず、都市空間そのものの変容が引き起こした歪みでもある。</t>
+          <t>この問題は、1人の勘違いだけでなく、街の作りそのものが変わってしまったことが原因でもあります。</t>
         </is>
       </c>
       <c r="D18" s="9">
@@ -1497,7 +1505,7 @@
       <c r="J18" s="14" t="n"/>
       <c r="K18" s="10" t="inlineStr">
         <is>
-          <t>都市のシルエットがパララックスで流れ、その上にジェネラティブな歪みが広がる。</t>
+          <t>街のシルエットがパララックスで流れ、その上にジェネラティブな歪みが広がる。</t>
         </is>
       </c>
       <c r="L18" s="10" t="n"/>
@@ -1508,12 +1516,12 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>② 公共空間の細分化</t>
+          <t>② 区切られた街</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>社会学者のエドワードソジャが1996年にロサンゼルスの都市再開発地区を調査した研究がある。</t>
+          <t>都市について研究していたエドワードソジャという学者が、1996年にロサンゼルスの街で調査を行いました。</t>
         </is>
       </c>
       <c r="D19" s="2">
@@ -1557,12 +1565,12 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>② 公共空間の細分化</t>
+          <t>② 区切られた街</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>公共広場をフェンスで囲い、入場料が必要な小規模ブース群へと分割した街区において、人々の行動変容を半年間にわたり定点観測した。</t>
+          <t>誰もが自由に使えた広場をフェンスで囲み、お金を払った人だけが入れる小さなブースに区切った場所で、半年間にわたって人々の様子を観察したのです。</t>
         </is>
       </c>
       <c r="D20" s="2">
@@ -1591,7 +1599,7 @@
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>広場の俯瞰図にフェンスの線が一筆書きで引かれ、格子状のブースに分割される。中を棒人間が動く。</t>
+          <t>広場の俯瞰図にフェンスの線が一筆書きで引かれ、格子状のブースに区切られる。中を棒人間が動く。</t>
         </is>
       </c>
       <c r="L20" s="3" t="n"/>
@@ -1602,12 +1610,12 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>② 公共空間の細分化</t>
+          <t>② 区切られた街</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>監視カメラの設置密度を高めたにもかかわらず、ブース内での規範逸脱行為は従来の公共空間の約3倍に達した。</t>
+          <t>防犯カメラをたくさん増やしたにもかかわらず、ブースの中でルールを破るいたずらや迷惑行為は、もとの広場の約3倍に増えてしまいました。</t>
         </is>
       </c>
       <c r="D21" s="2">
@@ -1640,12 +1648,12 @@
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>監視カメラのアイコンが次々に増える。横で「従来」と「ブース内」の棒グラフを比べ「約3倍」を表示。</t>
+          <t>防犯カメラのアイコンが次々に増える。横で「もとの広場」と「ブースの中」の棒グラフを比べ「約3倍」を表示。</t>
         </is>
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
-          <t>数値の出典が確認できていない。確認後にグラフ化する。</t>
+          <t>数値の出典が確認できていない。確認後にグラフにする。</t>
         </is>
       </c>
     </row>
@@ -1655,12 +1663,12 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>② 公共空間の細分化</t>
+          <t>② 区切られた街</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>公共空間の細分化と私有化は、共同体による自然な相互監視の目を無効化し、規律を内側から崩壊させる。</t>
+          <t>広場を細かく区切って個室にしてしまうと、お互いに見守り合う自然なブレーキが壊れてしまうのです。</t>
         </is>
       </c>
       <c r="D22" s="2">
@@ -1704,12 +1712,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>② 公共空間の細分化</t>
+          <t>② 区切られた街</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>かつて駅の待合所やベンチは、誰もが共有し、お互いの視線が交差するパブリックスペースだった。</t>
+          <t>昔の駅のベンチや待合室は、みんなで机や椅子を分け合い、お互いの目がある場所でした。</t>
         </is>
       </c>
       <c r="D23" s="2">
@@ -1753,12 +1761,12 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>② 公共空間の細分化</t>
+          <t>② 区切られた街</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>ところが、効率とプライバシーを追求した都市インフラは、共有地の中に「有料で孤立を買うカプセル」を埋め込み始めた。</t>
+          <t>ところが、便利さとプライバシーをどんどん進めた結果、街の共有スペースの中に「お金を払ってひとりぼっちになれるカプセル」が置かれるようになりました。</t>
         </is>
       </c>
       <c r="D24" s="2">
@@ -1802,12 +1810,12 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>② 公共空間の細分化</t>
+          <t>② 区切られた街</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>公共のルールと私室の自由が境界線上で衝突し、公衆道徳の抜け穴が駅のホームにぽっかりと口を開けているのだ。</t>
+          <t>みんなで使う場所のマナーと、自分の部屋のような自由さが狭いカプセルの中でぶつかり合って、大きな隙間が駅のホームに生まれてしまったのです。</t>
         </is>
       </c>
       <c r="D25" s="2">
@@ -1840,7 +1848,7 @@
       <c r="J25" s="7" t="n"/>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>「公共」と「私室」の領域がぶつかる図解。境界線がグリッチして裂け、穴が開く。</t>
+          <t>「みんなのマナー」と「自分の部屋の自由」の領域がぶつかる図解。境界線がグリッチして裂け、隙間が開く。</t>
         </is>
       </c>
       <c r="L25" s="3" t="n"/>
@@ -1856,7 +1864,7 @@
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>都市の合理化が皮肉にも公徳心を麻痺させたことは分かった。では、そもそもなぜその仕組みは必要とされたのか。</t>
+          <t>便利さを追い求めた仕組みが、皮肉にもみんなのモラルを麻痺させてしまったことは分かりました。では、そもそもなぜ私たちはそんな個室を必要としたのでしょうか。</t>
         </is>
       </c>
       <c r="D26" s="9">
@@ -1892,12 +1900,12 @@
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>③ 常時接続からの脱走</t>
+          <t>③ 繋がり疲れ</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>個室ブースでの逸脱は、単なる恥知らずの犯行ではなく、過剰に接続された現代社会からの暴力的な脱走劇である。</t>
+          <t>駅の小部屋で起きた事件は、ただの恥知らずな悪ふざけではなく、24時間スマホで誰かと繋がり続ける疲れから逃げ出そうとしたSOSでもありました。</t>
         </is>
       </c>
       <c r="D27" s="9">
@@ -1930,7 +1938,7 @@
       <c r="J27" s="14" t="n"/>
       <c r="K27" s="10" t="inlineStr">
         <is>
-          <t>パーティクルの接続線（見本03）が人物に絡みつく。「脱走劇」の文字が強く出る。</t>
+          <t>パーティクルの接続線（見本03）が人物に絡みつく。「SOS」の文字が点滅する。</t>
         </is>
       </c>
       <c r="L27" s="10" t="n"/>
@@ -1941,12 +1949,12 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>③ 常時接続からの脱走</t>
+          <t>③ 繋がり疲れ</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>社会学者のシェリータークルが2011年にビジネスパーソン200人を追跡した調査がある。</t>
+          <t>学者のシェリータークルが、2011年に働く大人200人を追いかけた調査があります。</t>
         </is>
       </c>
       <c r="D28" s="2">
@@ -1990,12 +1998,12 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>③ 常時接続からの脱走</t>
+          <t>③ 繋がり疲れ</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>常にスマートフォンで連絡を義務づけられた被験者に、1日1時間だけ通信を遮断した閉鎖空間を提供し、心理的変化を記録させた。</t>
+          <t>仕事の連絡をスマホでずっと受け続けなければいけない人たちを、1日1時間だけ通信を止めた閉まり切った部屋に入れて、どんな気持ちになるかを調べました。</t>
         </is>
       </c>
       <c r="D29" s="2">
@@ -2024,7 +2032,7 @@
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>スマホの通知バッジが増え続ける人物。閉鎖空間に入ると通知が止まり、1時間タイマーが動き出す。</t>
+          <t>スマホの通知バッジが増え続ける人物。部屋に入ると通知が止まり、1時間タイマーが動き出す。</t>
         </is>
       </c>
       <c r="L29" s="3" t="n"/>
@@ -2035,12 +2043,12 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>③ 常時接続からの脱走</t>
+          <t>③ 繋がり疲れ</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>追跡対象の約70パーセントが、社会的な規範意識よりも強烈な自己解放感を優先し、衝動的な行動を強く望んだ。</t>
+          <t>すると約70パーセントの人が、社会のルールを守ることよりも、誰にも邪魔されないすっきりした解放感を優先し、普段ならしないような衝動的な行動を強く望みました。</t>
         </is>
       </c>
       <c r="D30" s="2">
@@ -2069,12 +2077,12 @@
       <c r="J30" s="7" t="n"/>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>円グラフが70%まで伸び、「規範意識 &lt; 自己解放感」を天秤の図で添える。</t>
+          <t>円グラフが70%まで伸び、「ルール &lt; 解放感」を天秤の図で添える。</t>
         </is>
       </c>
       <c r="L30" s="8" t="inlineStr">
         <is>
-          <t>数値の出典が確認できていない。確認後にグラフ化する。</t>
+          <t>数値の出典が確認できていない。確認後にグラフにする。</t>
         </is>
       </c>
     </row>
@@ -2084,12 +2092,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>③ 常時接続からの脱走</t>
+          <t>③ 繋がり疲れ</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>常時接続の緊張から逃れる避難所を求めた人間は、規範そのものを脱ぎ捨てる。</t>
+          <t>繋がり続ける息苦しさから逃げ込める隠れ家を見つけたとき、人はマナーのブレーキまで一緒に外してしまうのです。</t>
         </is>
       </c>
       <c r="D31" s="2">
@@ -2118,14 +2126,10 @@
       <c r="J31" s="7" t="n"/>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>人物に絡んだ接続線が1本ずつ切れていき、人物が上着（＝規範の比喩）を脱ぎ落とす。</t>
-        </is>
-      </c>
-      <c r="L31" s="8" t="inlineStr">
-        <is>
-          <t>「脱ぎ捨てる」は比喩として描き、裸体は描かない。</t>
-        </is>
-      </c>
+          <t>人物に絡んだ接続線が1本ずつ切れていき、同時に「ブレーキ」のアイコンも外れて落ちる。</t>
+        </is>
+      </c>
+      <c r="L31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="9" t="n">
@@ -2138,7 +2142,7 @@
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>あの四角い箱は、監視と接続に疲れ果てた私たちが、群衆の中でプライベートを取り戻すために生み出した現代のシェルターだった。</t>
+          <t>あの駅の箱は、周りの目や連絡の通知に疲れ果てた私たちが、人混みの中でひとりきりになるために作った現代の隠れ家でした。</t>
         </is>
       </c>
       <c r="D32" s="9">
@@ -2187,7 +2191,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>あなたは、扉一枚で隔てられたその箱の中で、自分を完全にコントロールできると言い切れるだろうか。</t>
+          <t>あなたは、あの狭い箱に1人で入ったとき、絶対に自分をコントロールできると言い切れますか。</t>
         </is>
       </c>
       <c r="D33" s="2">
@@ -2281,7 +2285,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>密閉された小部屋に入ったとき、あなたならどんな衝動を感じるか、ぜひコメント欄で教えてほしい。</t>
+          <t>もしあなたが駅のあの個室に入ったら、どんな気分になるか、ぜひコメント欄で教えてください。</t>
         </is>
       </c>
       <c r="D35" s="2">
@@ -3170,7 +3174,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>ソジャはロサンゼルスを研究した実在の都市地理学者で、1996年に著書『Thirdspace』がある。ただし理論研究が中心で、こうした観測調査は確認できていない。「社会学者」という肩書きも一般的な紹介とは異なる。</t>
+          <t>ソジャはロサンゼルスを研究した実在の都市地理学者で、1996年に著書『Thirdspace』がある。ただし理論研究が中心で、こうした観測調査は確認できていない。</t>
         </is>
       </c>
       <c r="D4" s="19" t="inlineStr">

</xml_diff>